<commit_message>
Update stock_data and README
</commit_message>
<xml_diff>
--- a/stock_data.xlsx
+++ b/stock_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pushk\Desktop\COURSES\PROJECTS\EXCEL\stock portfolio tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F306A36-76DC-4AB5-86B7-A401874CBE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CAC464D-307E-46AB-BCD9-1FA44F9A3399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{C5389CB1-3F48-4573-9752-328BCB0657F4}"/>
   </bookViews>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="73">
   <si>
     <t>Ticker</t>
   </si>
@@ -302,13 +302,20 @@
   <si>
     <t>NSE Trading Portfolio Dashboard  ( 2022 - 2023)</t>
   </si>
+  <si>
+    <t>Initial Account Balance</t>
+  </si>
+  <si>
+    <t>₹5,00,000</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$₹-4009]\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -371,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -408,20 +415,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -430,6 +425,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6850,15 +6867,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>590550</xdr:colOff>
-      <xdr:row>0</xdr:row>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>180974</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>605789</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>5714</xdr:colOff>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6965,7 +6982,7 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
+      <xdr:colOff>952500</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
@@ -8423,11 +8440,11 @@
         <f t="shared" ref="R2:R29" si="5">(H2-F2)/F2</f>
         <v>0.11394901091918928</v>
       </c>
-      <c r="T2" s="15" t="s">
+      <c r="T2" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="U2" s="15"/>
-      <c r="V2" s="15"/>
+      <c r="U2" s="19"/>
+      <c r="V2" s="19"/>
       <c r="X2" s="2" t="str" cm="1">
         <f t="array" ref="X2:X9">_xlfn.UNIQUE(B2:B29)</f>
         <v>MARUTI.NS</v>
@@ -8711,11 +8728,11 @@
         <f t="shared" si="5"/>
         <v>-0.42770221904080163</v>
       </c>
-      <c r="T5" s="16" t="s">
+      <c r="T5" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="U5" s="16"/>
-      <c r="V5" s="16"/>
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
       <c r="W5" s="10"/>
       <c r="X5" s="2" t="str">
         <v>ZOMATO.NS</v>
@@ -8995,11 +9012,11 @@
         <f t="shared" si="5"/>
         <v>0.1812591508052708</v>
       </c>
-      <c r="T8" s="14" t="s">
+      <c r="T8" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="U8" s="14"/>
-      <c r="V8" s="14"/>
+      <c r="U8" s="20"/>
+      <c r="V8" s="20"/>
       <c r="W8"/>
       <c r="X8" s="2" t="str">
         <v>SUNPHARMA.NS</v>
@@ -9337,11 +9354,11 @@
         <f t="shared" si="5"/>
         <v>-5.1871511650599091E-2</v>
       </c>
-      <c r="T12" s="15" t="s">
+      <c r="T12" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="U12" s="15"/>
-      <c r="V12" s="15"/>
+      <c r="U12" s="19"/>
+      <c r="V12" s="19"/>
       <c r="X12" s="2" t="s">
         <v>46</v>
       </c>
@@ -9591,11 +9608,11 @@
         <f t="shared" si="5"/>
         <v>-0.10857086302454476</v>
       </c>
-      <c r="T15" s="14" t="s">
+      <c r="T15" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="U15" s="14"/>
-      <c r="V15" s="14"/>
+      <c r="U15" s="20"/>
+      <c r="V15" s="20"/>
       <c r="X15" s="2" t="str">
         <v>Finance</v>
       </c>
@@ -9843,11 +9860,11 @@
         <f t="shared" si="5"/>
         <v>0.15403802966842525</v>
       </c>
-      <c r="T18" s="15" t="s">
+      <c r="T18" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="U18" s="15"/>
-      <c r="V18" s="15"/>
+      <c r="U18" s="19"/>
+      <c r="V18" s="19"/>
       <c r="X18" s="2" t="str">
         <v>Metal</v>
       </c>
@@ -10085,11 +10102,11 @@
         <f t="shared" si="5"/>
         <v>-0.18842530282637954</v>
       </c>
-      <c r="T21" s="15" t="s">
+      <c r="T21" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="U21" s="15"/>
-      <c r="V21" s="15"/>
+      <c r="U21" s="19"/>
+      <c r="V21" s="19"/>
       <c r="AF21" s="4">
         <v>44928</v>
       </c>
@@ -10756,131 +10773,166 @@
   <dimension ref="A1:AC18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="7" width="8.88671875" style="13"/>
+    <col min="1" max="1" width="8.88671875" style="13"/>
+    <col min="2" max="2" width="11.6640625" style="13" customWidth="1"/>
+    <col min="3" max="7" width="8.88671875" style="13"/>
     <col min="8" max="8" width="8.88671875" style="13" customWidth="1"/>
     <col min="9" max="16384" width="8.88671875" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="J1" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="Q1" s="17" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="R1" s="17"/>
-      <c r="S1" s="17"/>
-      <c r="T1" s="17"/>
-      <c r="U1" s="17"/>
-      <c r="V1" s="17"/>
-      <c r="X1" s="17" t="s">
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="X1" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="Y1" s="17"/>
-      <c r="Z1" s="17"/>
-      <c r="AA1" s="17"/>
-      <c r="AB1" s="17"/>
-      <c r="AC1" s="17"/>
+      <c r="Y1" s="14"/>
+      <c r="Z1" s="14"/>
+      <c r="AA1" s="14"/>
+      <c r="AB1" s="14"/>
+      <c r="AC1" s="14"/>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="D2" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17" t="s">
+      <c r="E2" s="14"/>
+      <c r="G2" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17" t="s">
+      <c r="H2" s="14"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17" t="s">
+      <c r="K2" s="14"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="H2" s="17"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="22"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A3" s="19">
+      <c r="A3" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="25"/>
+      <c r="D3" s="15">
         <f>Analysis!T3</f>
         <v>19734.750000000029</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="20">
+      <c r="E3" s="15"/>
+      <c r="G3" s="16">
         <f>Analysis!T13</f>
         <v>0.5357142857142857</v>
       </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="20" t="str">
+      <c r="H3" s="16"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="16" t="str">
         <f>Analysis!T6</f>
         <v>ITC.NS (15.69%)</v>
       </c>
-      <c r="F3" s="21"/>
-      <c r="G3" s="21" t="str">
+      <c r="K3" s="16"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="17" t="str">
         <f>Analysis!T9</f>
         <v>FMCG- ₹17,844</v>
       </c>
-      <c r="H3" s="21"/>
+      <c r="N3" s="17"/>
+      <c r="O3" s="24"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A4" s="19"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="16"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="17"/>
+      <c r="O4" s="24"/>
     </row>
-    <row r="18" spans="3:15" x14ac:dyDescent="0.3">
-      <c r="C18" s="17" t="s">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+    </row>
+    <row r="18" spans="3:22" x14ac:dyDescent="0.3">
+      <c r="C18" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="J18" s="17" t="s">
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="J18" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="Q18" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="R18" s="18"/>
+      <c r="S18" s="18"/>
+      <c r="T18" s="18"/>
+      <c r="U18" s="18"/>
+      <c r="V18" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="16">
+    <mergeCell ref="J18:O18"/>
+    <mergeCell ref="Q18:V18"/>
+    <mergeCell ref="Q1:V1"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G3:H4"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J3:K4"/>
     <mergeCell ref="X1:AC1"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E4"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="M3:N4"/>
+    <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B4"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D4"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="E3:F4"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="G3:H4"/>
-    <mergeCell ref="J18:O18"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="J1:O1"/>
-    <mergeCell ref="Q1:V1"/>
-    <mergeCell ref="C18:H18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>